<commit_message>
feat: auto-expire bookings, delete validation, realtime seat hold, hold timer with pause/resume, payment flow fixes
- Auto-expire pending bookings after 10 minutes (cron + lazy cleanup)
- Block delete movie with future showtimes, concession with active bookings
- Realtime seat holding via seat_holds MySQL table + hold/release API endpoints
- Hold countdown timer: starts on seat select, persists across booking pages
- Timer pause/resume on QR payment open/cancel
- Cancel payment & QR timeout: release seats + full reset + navigate to seat selection
- Change payment method: resume hold timer
- Fix all TypeScript any warnings in PaymentPage with proper interfaces
</commit_message>
<xml_diff>
--- a/source-code/galaxy-cinema-hub-main/public/templates/movies_template.xlsx
+++ b/source-code/galaxy-cinema-hub-main/public/templates/movies_template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="28800" windowHeight="11460"/>
   </bookViews>
   <sheets>
     <sheet name="Movies" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Tên phim</t>
   </si>
@@ -62,31 +62,28 @@
     <t>Link Poster (URL)</t>
   </si>
   <si>
-    <t>Phim Mẫu 1</t>
-  </si>
-  <si>
-    <t>T16</t>
-  </si>
-  <si>
-    <t>Vietnam</t>
+    <t>Mặt Nạ Da Người</t>
+  </si>
+  <si>
+    <t>T18</t>
+  </si>
+  <si>
+    <t>International</t>
   </si>
   <si>
     <t>Coming Soon</t>
   </si>
   <si>
-    <t>Nguyễn Văn A</t>
-  </si>
-  <si>
-    <t>Trấn Thành, Lý Hải</t>
-  </si>
-  <si>
-    <t>2024-05-30</t>
-  </si>
-  <si>
-    <t>Mô tả nội dung phim...</t>
-  </si>
-  <si>
-    <t>https://youtube.com/...</t>
+    <t>Agus Riyanto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celine Evangelista, Djenar Maesa, Ayu Fajar Nugra </t>
+  </si>
+  <si>
+    <t>Ki Mangun Suroto là một nghệ nhân múa rối Wayang nổi tiếng và đầy tham vọng, ông khao khát nắm giữ tà thuật cổ xưa để đạt được sự giàu có và bất tử. Năm 2021, ông mời Citra làm nghệ sĩ hát Sinden trong một buổi lễ, nhưng thực chất là muốn cô trở thành vật tế cuối cùng. Trong khi cố gắng kiếm tiền chữa bệnh cho em gái, Citra dần bị cuốn vào những nghi lễ kinh hoàng và phải tìm cách thoát khỏi số phận đáng sợ của mình</t>
+  </si>
+  <si>
+    <t>https://youtu.be/JqOfZE0xa78?si=yo-yjAgTFGh5VrqS</t>
   </si>
   <si>
     <t>C:\Users\ACER\OneDrive\Pictures\Screenshots\Screenshot 2026-02-13 224052.png</t>
@@ -102,13 +99,19 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="12"/>
+  <fonts count="22">
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -565,153 +568,161 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -764,7 +775,7 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -907,7 +918,6 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
@@ -918,27 +928,31 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:tint val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -960,7 +974,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1018,7 +1032,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -1031,13 +1045,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
+                <a:tint val="80000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -1049,142 +1062,103 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="11.125" customWidth="1"/>
-    <col min="2" max="2" width="19.875" customWidth="1"/>
-    <col min="4" max="4" width="34.5" customWidth="1"/>
-    <col min="5" max="5" width="14.25" customWidth="1"/>
-    <col min="6" max="6" width="15.375" customWidth="1"/>
-    <col min="7" max="7" width="19.5" customWidth="1"/>
-    <col min="8" max="8" width="26.75" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="20.625" customWidth="1"/>
-    <col min="11" max="11" width="19.5" customWidth="1"/>
+    <col min="1" max="1" width="11.152380952381" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.8666666666667" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5809523809524" style="1" customWidth="1"/>
+    <col min="4" max="4" width="34.5809523809524" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.2952380952381" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.4380952380952" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.5809523809524" style="1" customWidth="1"/>
+    <col min="8" max="8" width="26.7238095238095" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17.0095238095238" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.5809523809524" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5809523809524" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" t="s">
+    <row r="1" ht="18.75" customHeight="1" spans="1:11">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" t="s">
+    <row r="2" ht="18.75" customHeight="1" spans="1:11">
+      <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2">
-        <v>120</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" s="3">
+        <v>86</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="4">
+        <v>46108</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="K2" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:K1 A2:J2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>